<commit_message>
Précisions sur les critère de recherche sur Coverage, DocumentReference et Encounter + nettoyage des fsh inutiles + précisions dans le narratif 048688c425fc1cd4a32610a99100b4f02f826192
</commit_message>
<xml_diff>
--- a/nmoreau/ig/StructureDefinition-preadmission-documentreference-fr.xlsx
+++ b/nmoreau/ig/StructureDefinition-preadmission-documentreference-fr.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-22T16:12:30+00:00</t>
+    <t>2025-05-26T06:59:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
-        <v>82</v>
+        <v>94</v>
       </c>
       <c r="G46" t="s" s="2">
         <v>94</v>

</xml_diff>